<commit_message>
feat: organização texto parte 2
</commit_message>
<xml_diff>
--- a/engstruct_casos.xlsx
+++ b/engstruct_casos.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Módulo de elasticidade médio à flexão (GPa) da longarina (GPa)</t>
+          <t>Módulo de elasticidade à flexão (GPa) da longarina (GPa)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -904,7 +904,7 @@
         <v>750</v>
       </c>
       <c r="Y3" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z3" t="n">
         <v>6</v>
@@ -916,7 +916,7 @@
         <v>750</v>
       </c>
       <c r="AC3" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD3" t="n">
         <v>30</v>
@@ -1212,7 +1212,7 @@
         <v>750</v>
       </c>
       <c r="Y5" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z5" t="n">
         <v>6</v>
@@ -1224,7 +1224,7 @@
         <v>750</v>
       </c>
       <c r="AC5" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD5" t="n">
         <v>30</v>
@@ -1520,7 +1520,7 @@
         <v>750</v>
       </c>
       <c r="Y7" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z7" t="n">
         <v>6</v>
@@ -1532,7 +1532,7 @@
         <v>750</v>
       </c>
       <c r="AC7" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD7" t="n">
         <v>30</v>
@@ -1828,7 +1828,7 @@
         <v>750</v>
       </c>
       <c r="Y9" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z9" t="n">
         <v>6</v>
@@ -1840,7 +1840,7 @@
         <v>750</v>
       </c>
       <c r="AC9" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD9" t="n">
         <v>30</v>
@@ -2136,7 +2136,7 @@
         <v>625</v>
       </c>
       <c r="Y11" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z11" t="n">
         <v>5</v>
@@ -2148,7 +2148,7 @@
         <v>625</v>
       </c>
       <c r="AC11" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD11" t="n">
         <v>30</v>
@@ -2444,7 +2444,7 @@
         <v>625</v>
       </c>
       <c r="Y13" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z13" t="n">
         <v>5</v>
@@ -2456,7 +2456,7 @@
         <v>625</v>
       </c>
       <c r="AC13" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD13" t="n">
         <v>30</v>
@@ -2752,7 +2752,7 @@
         <v>625</v>
       </c>
       <c r="Y15" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z15" t="n">
         <v>5</v>
@@ -2764,7 +2764,7 @@
         <v>625</v>
       </c>
       <c r="AC15" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD15" t="n">
         <v>30</v>
@@ -3060,7 +3060,7 @@
         <v>625</v>
       </c>
       <c r="Y17" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z17" t="n">
         <v>5</v>
@@ -3072,7 +3072,7 @@
         <v>625</v>
       </c>
       <c r="AC17" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD17" t="n">
         <v>30</v>
@@ -3368,7 +3368,7 @@
         <v>850</v>
       </c>
       <c r="Y19" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z19" t="n">
         <v>7</v>
@@ -3380,7 +3380,7 @@
         <v>850</v>
       </c>
       <c r="AC19" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD19" t="n">
         <v>30</v>
@@ -3676,7 +3676,7 @@
         <v>850</v>
       </c>
       <c r="Y21" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z21" t="n">
         <v>7</v>
@@ -3688,7 +3688,7 @@
         <v>850</v>
       </c>
       <c r="AC21" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD21" t="n">
         <v>30</v>
@@ -3984,7 +3984,7 @@
         <v>850</v>
       </c>
       <c r="Y23" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z23" t="n">
         <v>7</v>
@@ -3996,7 +3996,7 @@
         <v>850</v>
       </c>
       <c r="AC23" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD23" t="n">
         <v>30</v>
@@ -4292,7 +4292,7 @@
         <v>850</v>
       </c>
       <c r="Y25" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z25" t="n">
         <v>7</v>
@@ -4304,7 +4304,7 @@
         <v>850</v>
       </c>
       <c r="AC25" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD25" t="n">
         <v>30</v>
@@ -4600,7 +4600,7 @@
         <v>850</v>
       </c>
       <c r="Y27" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z27" t="n">
         <v>7</v>
@@ -4612,7 +4612,7 @@
         <v>850</v>
       </c>
       <c r="AC27" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD27" t="n">
         <v>30</v>
@@ -4908,7 +4908,7 @@
         <v>850</v>
       </c>
       <c r="Y29" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z29" t="n">
         <v>7</v>
@@ -4920,7 +4920,7 @@
         <v>850</v>
       </c>
       <c r="AC29" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD29" t="n">
         <v>30</v>
@@ -5216,7 +5216,7 @@
         <v>850</v>
       </c>
       <c r="Y31" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z31" t="n">
         <v>7</v>
@@ -5228,7 +5228,7 @@
         <v>850</v>
       </c>
       <c r="AC31" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD31" t="n">
         <v>30</v>
@@ -5524,7 +5524,7 @@
         <v>850</v>
       </c>
       <c r="Y33" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z33" t="n">
         <v>7</v>
@@ -5536,7 +5536,7 @@
         <v>850</v>
       </c>
       <c r="AC33" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD33" t="n">
         <v>30</v>
@@ -5832,7 +5832,7 @@
         <v>750</v>
       </c>
       <c r="Y35" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z35" t="n">
         <v>6</v>
@@ -5844,7 +5844,7 @@
         <v>750</v>
       </c>
       <c r="AC35" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD35" t="n">
         <v>30</v>
@@ -6140,7 +6140,7 @@
         <v>750</v>
       </c>
       <c r="Y37" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z37" t="n">
         <v>6</v>
@@ -6152,7 +6152,7 @@
         <v>750</v>
       </c>
       <c r="AC37" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD37" t="n">
         <v>30</v>
@@ -6448,7 +6448,7 @@
         <v>750</v>
       </c>
       <c r="Y39" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z39" t="n">
         <v>6</v>
@@ -6460,7 +6460,7 @@
         <v>750</v>
       </c>
       <c r="AC39" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD39" t="n">
         <v>30</v>
@@ -6756,7 +6756,7 @@
         <v>750</v>
       </c>
       <c r="Y41" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z41" t="n">
         <v>6</v>
@@ -6768,7 +6768,7 @@
         <v>750</v>
       </c>
       <c r="AC41" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD41" t="n">
         <v>30</v>
@@ -7064,7 +7064,7 @@
         <v>750</v>
       </c>
       <c r="Y43" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z43" t="n">
         <v>6</v>
@@ -7076,7 +7076,7 @@
         <v>750</v>
       </c>
       <c r="AC43" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD43" t="n">
         <v>30</v>
@@ -7372,7 +7372,7 @@
         <v>750</v>
       </c>
       <c r="Y45" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z45" t="n">
         <v>6</v>
@@ -7384,7 +7384,7 @@
         <v>750</v>
       </c>
       <c r="AC45" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD45" t="n">
         <v>30</v>
@@ -7680,7 +7680,7 @@
         <v>750</v>
       </c>
       <c r="Y47" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z47" t="n">
         <v>6</v>
@@ -7692,7 +7692,7 @@
         <v>750</v>
       </c>
       <c r="AC47" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD47" t="n">
         <v>30</v>
@@ -7988,7 +7988,7 @@
         <v>750</v>
       </c>
       <c r="Y49" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z49" t="n">
         <v>6</v>
@@ -8000,7 +8000,7 @@
         <v>750</v>
       </c>
       <c r="AC49" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD49" t="n">
         <v>30</v>
@@ -8296,7 +8296,7 @@
         <v>850</v>
       </c>
       <c r="Y51" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z51" t="n">
         <v>7</v>
@@ -8308,7 +8308,7 @@
         <v>850</v>
       </c>
       <c r="AC51" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD51" t="n">
         <v>30</v>
@@ -8604,7 +8604,7 @@
         <v>850</v>
       </c>
       <c r="Y53" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z53" t="n">
         <v>7</v>
@@ -8616,7 +8616,7 @@
         <v>850</v>
       </c>
       <c r="AC53" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD53" t="n">
         <v>30</v>
@@ -8912,7 +8912,7 @@
         <v>850</v>
       </c>
       <c r="Y55" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z55" t="n">
         <v>7</v>
@@ -8924,7 +8924,7 @@
         <v>850</v>
       </c>
       <c r="AC55" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD55" t="n">
         <v>30</v>
@@ -9220,7 +9220,7 @@
         <v>850</v>
       </c>
       <c r="Y57" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z57" t="n">
         <v>7</v>
@@ -9232,7 +9232,7 @@
         <v>850</v>
       </c>
       <c r="AC57" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD57" t="n">
         <v>30</v>
@@ -9528,7 +9528,7 @@
         <v>625</v>
       </c>
       <c r="Y59" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z59" t="n">
         <v>5</v>
@@ -9540,7 +9540,7 @@
         <v>625</v>
       </c>
       <c r="AC59" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD59" t="n">
         <v>30</v>
@@ -9836,7 +9836,7 @@
         <v>625</v>
       </c>
       <c r="Y61" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z61" t="n">
         <v>5</v>
@@ -9848,7 +9848,7 @@
         <v>625</v>
       </c>
       <c r="AC61" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD61" t="n">
         <v>30</v>
@@ -10144,7 +10144,7 @@
         <v>625</v>
       </c>
       <c r="Y63" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z63" t="n">
         <v>5</v>
@@ -10156,7 +10156,7 @@
         <v>625</v>
       </c>
       <c r="AC63" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD63" t="n">
         <v>30</v>
@@ -10452,7 +10452,7 @@
         <v>625</v>
       </c>
       <c r="Y65" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z65" t="n">
         <v>5</v>
@@ -10464,7 +10464,7 @@
         <v>625</v>
       </c>
       <c r="AC65" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD65" t="n">
         <v>30</v>
@@ -10760,7 +10760,7 @@
         <v>750</v>
       </c>
       <c r="Y67" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z67" t="n">
         <v>6</v>
@@ -10772,7 +10772,7 @@
         <v>750</v>
       </c>
       <c r="AC67" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD67" t="n">
         <v>30</v>
@@ -11068,7 +11068,7 @@
         <v>750</v>
       </c>
       <c r="Y69" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z69" t="n">
         <v>6</v>
@@ -11080,7 +11080,7 @@
         <v>750</v>
       </c>
       <c r="AC69" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD69" t="n">
         <v>30</v>
@@ -11376,7 +11376,7 @@
         <v>750</v>
       </c>
       <c r="Y71" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z71" t="n">
         <v>6</v>
@@ -11388,7 +11388,7 @@
         <v>750</v>
       </c>
       <c r="AC71" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD71" t="n">
         <v>30</v>
@@ -11684,7 +11684,7 @@
         <v>750</v>
       </c>
       <c r="Y73" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z73" t="n">
         <v>6</v>
@@ -11696,7 +11696,7 @@
         <v>750</v>
       </c>
       <c r="AC73" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD73" t="n">
         <v>30</v>
@@ -11992,7 +11992,7 @@
         <v>625</v>
       </c>
       <c r="Y75" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z75" t="n">
         <v>5</v>
@@ -12004,7 +12004,7 @@
         <v>625</v>
       </c>
       <c r="AC75" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD75" t="n">
         <v>30</v>
@@ -12300,7 +12300,7 @@
         <v>625</v>
       </c>
       <c r="Y77" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z77" t="n">
         <v>5</v>
@@ -12312,7 +12312,7 @@
         <v>625</v>
       </c>
       <c r="AC77" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD77" t="n">
         <v>30</v>
@@ -12608,7 +12608,7 @@
         <v>625</v>
       </c>
       <c r="Y79" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z79" t="n">
         <v>5</v>
@@ -12620,7 +12620,7 @@
         <v>625</v>
       </c>
       <c r="AC79" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD79" t="n">
         <v>30</v>
@@ -12916,7 +12916,7 @@
         <v>625</v>
       </c>
       <c r="Y81" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z81" t="n">
         <v>5</v>
@@ -12928,7 +12928,7 @@
         <v>625</v>
       </c>
       <c r="AC81" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD81" t="n">
         <v>30</v>
@@ -13224,7 +13224,7 @@
         <v>625</v>
       </c>
       <c r="Y83" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z83" t="n">
         <v>5</v>
@@ -13236,7 +13236,7 @@
         <v>625</v>
       </c>
       <c r="AC83" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD83" t="n">
         <v>30</v>
@@ -13532,7 +13532,7 @@
         <v>625</v>
       </c>
       <c r="Y85" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z85" t="n">
         <v>5</v>
@@ -13544,7 +13544,7 @@
         <v>625</v>
       </c>
       <c r="AC85" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD85" t="n">
         <v>30</v>
@@ -13840,7 +13840,7 @@
         <v>625</v>
       </c>
       <c r="Y87" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z87" t="n">
         <v>5</v>
@@ -13852,7 +13852,7 @@
         <v>625</v>
       </c>
       <c r="AC87" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD87" t="n">
         <v>30</v>
@@ -14148,7 +14148,7 @@
         <v>625</v>
       </c>
       <c r="Y89" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z89" t="n">
         <v>5</v>
@@ -14160,7 +14160,7 @@
         <v>625</v>
       </c>
       <c r="AC89" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD89" t="n">
         <v>30</v>
@@ -14456,7 +14456,7 @@
         <v>625</v>
       </c>
       <c r="Y91" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z91" t="n">
         <v>5</v>
@@ -14468,7 +14468,7 @@
         <v>625</v>
       </c>
       <c r="AC91" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD91" t="n">
         <v>30</v>
@@ -14764,7 +14764,7 @@
         <v>625</v>
       </c>
       <c r="Y93" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z93" t="n">
         <v>5</v>
@@ -14776,7 +14776,7 @@
         <v>625</v>
       </c>
       <c r="AC93" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD93" t="n">
         <v>30</v>
@@ -15072,7 +15072,7 @@
         <v>625</v>
       </c>
       <c r="Y95" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z95" t="n">
         <v>5</v>
@@ -15084,7 +15084,7 @@
         <v>625</v>
       </c>
       <c r="AC95" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD95" t="n">
         <v>30</v>
@@ -15380,7 +15380,7 @@
         <v>625</v>
       </c>
       <c r="Y97" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z97" t="n">
         <v>5</v>
@@ -15392,7 +15392,7 @@
         <v>625</v>
       </c>
       <c r="AC97" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD97" t="n">
         <v>30</v>
@@ -15688,7 +15688,7 @@
         <v>625</v>
       </c>
       <c r="Y99" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z99" t="n">
         <v>5</v>
@@ -15700,7 +15700,7 @@
         <v>625</v>
       </c>
       <c r="AC99" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD99" t="n">
         <v>30</v>
@@ -15996,7 +15996,7 @@
         <v>625</v>
       </c>
       <c r="Y101" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z101" t="n">
         <v>5</v>
@@ -16008,7 +16008,7 @@
         <v>625</v>
       </c>
       <c r="AC101" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD101" t="n">
         <v>30</v>
@@ -16304,7 +16304,7 @@
         <v>625</v>
       </c>
       <c r="Y103" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z103" t="n">
         <v>5</v>
@@ -16316,7 +16316,7 @@
         <v>625</v>
       </c>
       <c r="AC103" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD103" t="n">
         <v>30</v>
@@ -16612,7 +16612,7 @@
         <v>625</v>
       </c>
       <c r="Y105" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z105" t="n">
         <v>5</v>
@@ -16624,7 +16624,7 @@
         <v>625</v>
       </c>
       <c r="AC105" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD105" t="n">
         <v>30</v>
@@ -16920,7 +16920,7 @@
         <v>500</v>
       </c>
       <c r="Y107" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z107" t="n">
         <v>4</v>
@@ -16932,7 +16932,7 @@
         <v>500</v>
       </c>
       <c r="AC107" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD107" t="n">
         <v>30</v>
@@ -17228,7 +17228,7 @@
         <v>500</v>
       </c>
       <c r="Y109" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z109" t="n">
         <v>4</v>
@@ -17240,7 +17240,7 @@
         <v>500</v>
       </c>
       <c r="AC109" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD109" t="n">
         <v>30</v>
@@ -17536,7 +17536,7 @@
         <v>500</v>
       </c>
       <c r="Y111" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z111" t="n">
         <v>4</v>
@@ -17548,7 +17548,7 @@
         <v>500</v>
       </c>
       <c r="AC111" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD111" t="n">
         <v>30</v>
@@ -17844,7 +17844,7 @@
         <v>500</v>
       </c>
       <c r="Y113" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z113" t="n">
         <v>4</v>
@@ -17856,7 +17856,7 @@
         <v>500</v>
       </c>
       <c r="AC113" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD113" t="n">
         <v>30</v>
@@ -18152,7 +18152,7 @@
         <v>500</v>
       </c>
       <c r="Y115" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z115" t="n">
         <v>4</v>
@@ -18164,7 +18164,7 @@
         <v>500</v>
       </c>
       <c r="AC115" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD115" t="n">
         <v>30</v>
@@ -18460,7 +18460,7 @@
         <v>500</v>
       </c>
       <c r="Y117" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z117" t="n">
         <v>4</v>
@@ -18472,7 +18472,7 @@
         <v>500</v>
       </c>
       <c r="AC117" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD117" t="n">
         <v>30</v>
@@ -18768,7 +18768,7 @@
         <v>500</v>
       </c>
       <c r="Y119" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z119" t="n">
         <v>4</v>
@@ -18780,7 +18780,7 @@
         <v>500</v>
       </c>
       <c r="AC119" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD119" t="n">
         <v>30</v>
@@ -19076,7 +19076,7 @@
         <v>500</v>
       </c>
       <c r="Y121" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z121" t="n">
         <v>4</v>
@@ -19088,7 +19088,7 @@
         <v>500</v>
       </c>
       <c r="AC121" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD121" t="n">
         <v>30</v>
@@ -19384,7 +19384,7 @@
         <v>500</v>
       </c>
       <c r="Y123" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z123" t="n">
         <v>4</v>
@@ -19396,7 +19396,7 @@
         <v>500</v>
       </c>
       <c r="AC123" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD123" t="n">
         <v>30</v>
@@ -19692,7 +19692,7 @@
         <v>500</v>
       </c>
       <c r="Y125" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z125" t="n">
         <v>4</v>
@@ -19704,7 +19704,7 @@
         <v>500</v>
       </c>
       <c r="AC125" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD125" t="n">
         <v>30</v>
@@ -20000,7 +20000,7 @@
         <v>500</v>
       </c>
       <c r="Y127" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z127" t="n">
         <v>4</v>
@@ -20012,7 +20012,7 @@
         <v>500</v>
       </c>
       <c r="AC127" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD127" t="n">
         <v>30</v>
@@ -20308,7 +20308,7 @@
         <v>500</v>
       </c>
       <c r="Y129" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z129" t="n">
         <v>4</v>
@@ -20320,7 +20320,7 @@
         <v>500</v>
       </c>
       <c r="AC129" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD129" t="n">
         <v>30</v>
@@ -20616,7 +20616,7 @@
         <v>1000</v>
       </c>
       <c r="Y131" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z131" t="n">
         <v>8</v>
@@ -20628,7 +20628,7 @@
         <v>1000</v>
       </c>
       <c r="AC131" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD131" t="n">
         <v>30</v>
@@ -20924,7 +20924,7 @@
         <v>1000</v>
       </c>
       <c r="Y133" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z133" t="n">
         <v>8</v>
@@ -20936,7 +20936,7 @@
         <v>1000</v>
       </c>
       <c r="AC133" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD133" t="n">
         <v>30</v>
@@ -21232,7 +21232,7 @@
         <v>1000</v>
       </c>
       <c r="Y135" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z135" t="n">
         <v>8</v>
@@ -21244,7 +21244,7 @@
         <v>1000</v>
       </c>
       <c r="AC135" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD135" t="n">
         <v>30</v>
@@ -21540,7 +21540,7 @@
         <v>1000</v>
       </c>
       <c r="Y137" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z137" t="n">
         <v>8</v>
@@ -21552,7 +21552,7 @@
         <v>1000</v>
       </c>
       <c r="AC137" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD137" t="n">
         <v>30</v>
@@ -21848,7 +21848,7 @@
         <v>625</v>
       </c>
       <c r="Y139" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z139" t="n">
         <v>5</v>
@@ -21860,7 +21860,7 @@
         <v>625</v>
       </c>
       <c r="AC139" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD139" t="n">
         <v>30</v>
@@ -22156,7 +22156,7 @@
         <v>625</v>
       </c>
       <c r="Y141" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z141" t="n">
         <v>5</v>
@@ -22168,7 +22168,7 @@
         <v>625</v>
       </c>
       <c r="AC141" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD141" t="n">
         <v>30</v>
@@ -22464,7 +22464,7 @@
         <v>625</v>
       </c>
       <c r="Y143" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z143" t="n">
         <v>5</v>
@@ -22476,7 +22476,7 @@
         <v>625</v>
       </c>
       <c r="AC143" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD143" t="n">
         <v>30</v>
@@ -22772,7 +22772,7 @@
         <v>625</v>
       </c>
       <c r="Y145" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z145" t="n">
         <v>5</v>
@@ -22784,7 +22784,7 @@
         <v>625</v>
       </c>
       <c r="AC145" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD145" t="n">
         <v>30</v>
@@ -23080,7 +23080,7 @@
         <v>625</v>
       </c>
       <c r="Y147" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z147" t="n">
         <v>5</v>
@@ -23092,7 +23092,7 @@
         <v>625</v>
       </c>
       <c r="AC147" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD147" t="n">
         <v>30</v>
@@ -23388,7 +23388,7 @@
         <v>625</v>
       </c>
       <c r="Y149" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z149" t="n">
         <v>5</v>
@@ -23400,7 +23400,7 @@
         <v>625</v>
       </c>
       <c r="AC149" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD149" t="n">
         <v>30</v>
@@ -23696,7 +23696,7 @@
         <v>625</v>
       </c>
       <c r="Y151" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z151" t="n">
         <v>5</v>
@@ -23708,7 +23708,7 @@
         <v>625</v>
       </c>
       <c r="AC151" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD151" t="n">
         <v>30</v>
@@ -24004,7 +24004,7 @@
         <v>625</v>
       </c>
       <c r="Y153" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z153" t="n">
         <v>5</v>
@@ -24016,7 +24016,7 @@
         <v>625</v>
       </c>
       <c r="AC153" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD153" t="n">
         <v>30</v>
@@ -24312,7 +24312,7 @@
         <v>850</v>
       </c>
       <c r="Y155" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z155" t="n">
         <v>7</v>
@@ -24324,7 +24324,7 @@
         <v>850</v>
       </c>
       <c r="AC155" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD155" t="n">
         <v>30</v>
@@ -24620,7 +24620,7 @@
         <v>850</v>
       </c>
       <c r="Y157" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z157" t="n">
         <v>7</v>
@@ -24632,7 +24632,7 @@
         <v>850</v>
       </c>
       <c r="AC157" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD157" t="n">
         <v>30</v>
@@ -24928,7 +24928,7 @@
         <v>850</v>
       </c>
       <c r="Y159" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z159" t="n">
         <v>7</v>
@@ -24940,7 +24940,7 @@
         <v>850</v>
       </c>
       <c r="AC159" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD159" t="n">
         <v>30</v>
@@ -25236,7 +25236,7 @@
         <v>850</v>
       </c>
       <c r="Y161" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z161" t="n">
         <v>7</v>
@@ -25248,7 +25248,7 @@
         <v>850</v>
       </c>
       <c r="AC161" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD161" t="n">
         <v>30</v>
@@ -25544,7 +25544,7 @@
         <v>850</v>
       </c>
       <c r="Y163" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z163" t="n">
         <v>7</v>
@@ -25556,7 +25556,7 @@
         <v>850</v>
       </c>
       <c r="AC163" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD163" t="n">
         <v>30</v>
@@ -25852,7 +25852,7 @@
         <v>850</v>
       </c>
       <c r="Y165" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z165" t="n">
         <v>7</v>
@@ -25864,7 +25864,7 @@
         <v>850</v>
       </c>
       <c r="AC165" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD165" t="n">
         <v>30</v>
@@ -26160,7 +26160,7 @@
         <v>850</v>
       </c>
       <c r="Y167" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z167" t="n">
         <v>7</v>
@@ -26172,7 +26172,7 @@
         <v>850</v>
       </c>
       <c r="AC167" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD167" t="n">
         <v>30</v>
@@ -26468,7 +26468,7 @@
         <v>850</v>
       </c>
       <c r="Y169" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z169" t="n">
         <v>7</v>
@@ -26480,7 +26480,7 @@
         <v>850</v>
       </c>
       <c r="AC169" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD169" t="n">
         <v>30</v>
@@ -26776,7 +26776,7 @@
         <v>625</v>
       </c>
       <c r="Y171" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z171" t="n">
         <v>5</v>
@@ -26788,7 +26788,7 @@
         <v>625</v>
       </c>
       <c r="AC171" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD171" t="n">
         <v>30</v>
@@ -27084,7 +27084,7 @@
         <v>625</v>
       </c>
       <c r="Y173" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z173" t="n">
         <v>5</v>
@@ -27096,7 +27096,7 @@
         <v>625</v>
       </c>
       <c r="AC173" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD173" t="n">
         <v>30</v>
@@ -27392,7 +27392,7 @@
         <v>625</v>
       </c>
       <c r="Y175" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z175" t="n">
         <v>5</v>
@@ -27404,7 +27404,7 @@
         <v>625</v>
       </c>
       <c r="AC175" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD175" t="n">
         <v>30</v>
@@ -27700,7 +27700,7 @@
         <v>625</v>
       </c>
       <c r="Y177" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z177" t="n">
         <v>5</v>
@@ -27712,7 +27712,7 @@
         <v>625</v>
       </c>
       <c r="AC177" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD177" t="n">
         <v>30</v>
@@ -28008,7 +28008,7 @@
         <v>750</v>
       </c>
       <c r="Y179" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z179" t="n">
         <v>6</v>
@@ -28020,7 +28020,7 @@
         <v>750</v>
       </c>
       <c r="AC179" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD179" t="n">
         <v>30</v>
@@ -28316,7 +28316,7 @@
         <v>750</v>
       </c>
       <c r="Y181" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z181" t="n">
         <v>6</v>
@@ -28328,7 +28328,7 @@
         <v>750</v>
       </c>
       <c r="AC181" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD181" t="n">
         <v>30</v>
@@ -28624,7 +28624,7 @@
         <v>750</v>
       </c>
       <c r="Y183" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z183" t="n">
         <v>6</v>
@@ -28636,7 +28636,7 @@
         <v>750</v>
       </c>
       <c r="AC183" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD183" t="n">
         <v>30</v>
@@ -28932,7 +28932,7 @@
         <v>750</v>
       </c>
       <c r="Y185" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z185" t="n">
         <v>6</v>
@@ -28944,7 +28944,7 @@
         <v>750</v>
       </c>
       <c r="AC185" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD185" t="n">
         <v>30</v>
@@ -29240,7 +29240,7 @@
         <v>750</v>
       </c>
       <c r="Y187" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z187" t="n">
         <v>6</v>
@@ -29252,7 +29252,7 @@
         <v>750</v>
       </c>
       <c r="AC187" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD187" t="n">
         <v>30</v>
@@ -29548,7 +29548,7 @@
         <v>750</v>
       </c>
       <c r="Y189" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z189" t="n">
         <v>6</v>
@@ -29560,7 +29560,7 @@
         <v>750</v>
       </c>
       <c r="AC189" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD189" t="n">
         <v>30</v>
@@ -29856,7 +29856,7 @@
         <v>750</v>
       </c>
       <c r="Y191" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z191" t="n">
         <v>6</v>
@@ -29868,7 +29868,7 @@
         <v>750</v>
       </c>
       <c r="AC191" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD191" t="n">
         <v>30</v>
@@ -30164,7 +30164,7 @@
         <v>750</v>
       </c>
       <c r="Y193" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z193" t="n">
         <v>6</v>
@@ -30176,7 +30176,7 @@
         <v>750</v>
       </c>
       <c r="AC193" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD193" t="n">
         <v>30</v>
@@ -30472,7 +30472,7 @@
         <v>850</v>
       </c>
       <c r="Y195" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z195" t="n">
         <v>7</v>
@@ -30484,7 +30484,7 @@
         <v>850</v>
       </c>
       <c r="AC195" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD195" t="n">
         <v>30</v>
@@ -30780,7 +30780,7 @@
         <v>850</v>
       </c>
       <c r="Y197" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z197" t="n">
         <v>7</v>
@@ -30792,7 +30792,7 @@
         <v>850</v>
       </c>
       <c r="AC197" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD197" t="n">
         <v>30</v>
@@ -31088,7 +31088,7 @@
         <v>850</v>
       </c>
       <c r="Y199" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z199" t="n">
         <v>7</v>
@@ -31100,7 +31100,7 @@
         <v>850</v>
       </c>
       <c r="AC199" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD199" t="n">
         <v>30</v>
@@ -31396,7 +31396,7 @@
         <v>850</v>
       </c>
       <c r="Y201" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z201" t="n">
         <v>7</v>
@@ -31408,7 +31408,7 @@
         <v>850</v>
       </c>
       <c r="AC201" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD201" t="n">
         <v>30</v>
@@ -31704,7 +31704,7 @@
         <v>750</v>
       </c>
       <c r="Y203" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z203" t="n">
         <v>6</v>
@@ -31716,7 +31716,7 @@
         <v>750</v>
       </c>
       <c r="AC203" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD203" t="n">
         <v>30</v>
@@ -32012,7 +32012,7 @@
         <v>750</v>
       </c>
       <c r="Y205" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z205" t="n">
         <v>6</v>
@@ -32024,7 +32024,7 @@
         <v>750</v>
       </c>
       <c r="AC205" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD205" t="n">
         <v>30</v>
@@ -32320,7 +32320,7 @@
         <v>750</v>
       </c>
       <c r="Y207" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z207" t="n">
         <v>6</v>
@@ -32332,7 +32332,7 @@
         <v>750</v>
       </c>
       <c r="AC207" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD207" t="n">
         <v>30</v>
@@ -32628,7 +32628,7 @@
         <v>750</v>
       </c>
       <c r="Y209" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z209" t="n">
         <v>6</v>
@@ -32640,7 +32640,7 @@
         <v>750</v>
       </c>
       <c r="AC209" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD209" t="n">
         <v>30</v>
@@ -32936,7 +32936,7 @@
         <v>1000</v>
       </c>
       <c r="Y211" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z211" t="n">
         <v>8</v>
@@ -32948,7 +32948,7 @@
         <v>1000</v>
       </c>
       <c r="AC211" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD211" t="n">
         <v>30</v>
@@ -33244,7 +33244,7 @@
         <v>1000</v>
       </c>
       <c r="Y213" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z213" t="n">
         <v>8</v>
@@ -33256,7 +33256,7 @@
         <v>1000</v>
       </c>
       <c r="AC213" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD213" t="n">
         <v>30</v>
@@ -33552,7 +33552,7 @@
         <v>1000</v>
       </c>
       <c r="Y215" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z215" t="n">
         <v>8</v>
@@ -33564,7 +33564,7 @@
         <v>1000</v>
       </c>
       <c r="AC215" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD215" t="n">
         <v>30</v>
@@ -33860,7 +33860,7 @@
         <v>1000</v>
       </c>
       <c r="Y217" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z217" t="n">
         <v>8</v>
@@ -33872,7 +33872,7 @@
         <v>1000</v>
       </c>
       <c r="AC217" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD217" t="n">
         <v>30</v>
@@ -34168,7 +34168,7 @@
         <v>625</v>
       </c>
       <c r="Y219" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z219" t="n">
         <v>5</v>
@@ -34180,7 +34180,7 @@
         <v>625</v>
       </c>
       <c r="AC219" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD219" t="n">
         <v>30</v>
@@ -34476,7 +34476,7 @@
         <v>625</v>
       </c>
       <c r="Y221" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z221" t="n">
         <v>5</v>
@@ -34488,7 +34488,7 @@
         <v>625</v>
       </c>
       <c r="AC221" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD221" t="n">
         <v>30</v>
@@ -34784,7 +34784,7 @@
         <v>625</v>
       </c>
       <c r="Y223" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z223" t="n">
         <v>5</v>
@@ -34796,7 +34796,7 @@
         <v>625</v>
       </c>
       <c r="AC223" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD223" t="n">
         <v>30</v>
@@ -35092,7 +35092,7 @@
         <v>625</v>
       </c>
       <c r="Y225" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z225" t="n">
         <v>5</v>
@@ -35104,7 +35104,7 @@
         <v>625</v>
       </c>
       <c r="AC225" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD225" t="n">
         <v>30</v>
@@ -35400,7 +35400,7 @@
         <v>850</v>
       </c>
       <c r="Y227" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z227" t="n">
         <v>7</v>
@@ -35412,7 +35412,7 @@
         <v>850</v>
       </c>
       <c r="AC227" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD227" t="n">
         <v>30</v>
@@ -35708,7 +35708,7 @@
         <v>850</v>
       </c>
       <c r="Y229" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z229" t="n">
         <v>7</v>
@@ -35720,7 +35720,7 @@
         <v>850</v>
       </c>
       <c r="AC229" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD229" t="n">
         <v>30</v>
@@ -36016,7 +36016,7 @@
         <v>850</v>
       </c>
       <c r="Y231" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z231" t="n">
         <v>7</v>
@@ -36028,7 +36028,7 @@
         <v>850</v>
       </c>
       <c r="AC231" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD231" t="n">
         <v>30</v>
@@ -36324,7 +36324,7 @@
         <v>850</v>
       </c>
       <c r="Y233" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z233" t="n">
         <v>7</v>
@@ -36336,7 +36336,7 @@
         <v>850</v>
       </c>
       <c r="AC233" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD233" t="n">
         <v>30</v>
@@ -36632,7 +36632,7 @@
         <v>750</v>
       </c>
       <c r="Y235" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z235" t="n">
         <v>6</v>
@@ -36644,7 +36644,7 @@
         <v>750</v>
       </c>
       <c r="AC235" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD235" t="n">
         <v>30</v>
@@ -36940,7 +36940,7 @@
         <v>750</v>
       </c>
       <c r="Y237" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z237" t="n">
         <v>6</v>
@@ -36952,7 +36952,7 @@
         <v>750</v>
       </c>
       <c r="AC237" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD237" t="n">
         <v>30</v>
@@ -37248,7 +37248,7 @@
         <v>750</v>
       </c>
       <c r="Y239" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z239" t="n">
         <v>6</v>
@@ -37260,7 +37260,7 @@
         <v>750</v>
       </c>
       <c r="AC239" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD239" t="n">
         <v>30</v>
@@ -37556,7 +37556,7 @@
         <v>750</v>
       </c>
       <c r="Y241" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z241" t="n">
         <v>6</v>
@@ -37568,7 +37568,7 @@
         <v>750</v>
       </c>
       <c r="AC241" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD241" t="n">
         <v>30</v>
@@ -37864,7 +37864,7 @@
         <v>750</v>
       </c>
       <c r="Y243" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z243" t="n">
         <v>6</v>
@@ -37876,7 +37876,7 @@
         <v>750</v>
       </c>
       <c r="AC243" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD243" t="n">
         <v>30</v>
@@ -38172,7 +38172,7 @@
         <v>750</v>
       </c>
       <c r="Y245" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z245" t="n">
         <v>6</v>
@@ -38184,7 +38184,7 @@
         <v>750</v>
       </c>
       <c r="AC245" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD245" t="n">
         <v>30</v>
@@ -38480,7 +38480,7 @@
         <v>750</v>
       </c>
       <c r="Y247" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z247" t="n">
         <v>6</v>
@@ -38492,7 +38492,7 @@
         <v>750</v>
       </c>
       <c r="AC247" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD247" t="n">
         <v>30</v>
@@ -38788,7 +38788,7 @@
         <v>750</v>
       </c>
       <c r="Y249" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z249" t="n">
         <v>6</v>
@@ -38800,7 +38800,7 @@
         <v>750</v>
       </c>
       <c r="AC249" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD249" t="n">
         <v>30</v>
@@ -39096,7 +39096,7 @@
         <v>850</v>
       </c>
       <c r="Y251" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z251" t="n">
         <v>7</v>
@@ -39108,7 +39108,7 @@
         <v>850</v>
       </c>
       <c r="AC251" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD251" t="n">
         <v>30</v>
@@ -39404,7 +39404,7 @@
         <v>850</v>
       </c>
       <c r="Y253" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z253" t="n">
         <v>7</v>
@@ -39416,7 +39416,7 @@
         <v>850</v>
       </c>
       <c r="AC253" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD253" t="n">
         <v>30</v>
@@ -39712,7 +39712,7 @@
         <v>850</v>
       </c>
       <c r="Y255" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z255" t="n">
         <v>7</v>
@@ -39724,7 +39724,7 @@
         <v>850</v>
       </c>
       <c r="AC255" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD255" t="n">
         <v>30</v>
@@ -40020,7 +40020,7 @@
         <v>850</v>
       </c>
       <c r="Y257" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z257" t="n">
         <v>7</v>
@@ -40032,7 +40032,7 @@
         <v>850</v>
       </c>
       <c r="AC257" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD257" t="n">
         <v>30</v>
@@ -40328,7 +40328,7 @@
         <v>750</v>
       </c>
       <c r="Y259" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z259" t="n">
         <v>6</v>
@@ -40340,7 +40340,7 @@
         <v>750</v>
       </c>
       <c r="AC259" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD259" t="n">
         <v>30</v>
@@ -40636,7 +40636,7 @@
         <v>750</v>
       </c>
       <c r="Y261" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z261" t="n">
         <v>6</v>
@@ -40648,7 +40648,7 @@
         <v>750</v>
       </c>
       <c r="AC261" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD261" t="n">
         <v>30</v>
@@ -40944,7 +40944,7 @@
         <v>750</v>
       </c>
       <c r="Y263" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z263" t="n">
         <v>6</v>
@@ -40956,7 +40956,7 @@
         <v>750</v>
       </c>
       <c r="AC263" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD263" t="n">
         <v>30</v>
@@ -41252,7 +41252,7 @@
         <v>750</v>
       </c>
       <c r="Y265" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z265" t="n">
         <v>6</v>
@@ -41264,7 +41264,7 @@
         <v>750</v>
       </c>
       <c r="AC265" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD265" t="n">
         <v>30</v>
@@ -41560,7 +41560,7 @@
         <v>750</v>
       </c>
       <c r="Y267" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z267" t="n">
         <v>6</v>
@@ -41572,7 +41572,7 @@
         <v>750</v>
       </c>
       <c r="AC267" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD267" t="n">
         <v>30</v>
@@ -41868,7 +41868,7 @@
         <v>750</v>
       </c>
       <c r="Y269" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z269" t="n">
         <v>6</v>
@@ -41880,7 +41880,7 @@
         <v>750</v>
       </c>
       <c r="AC269" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD269" t="n">
         <v>30</v>
@@ -42176,7 +42176,7 @@
         <v>750</v>
       </c>
       <c r="Y271" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z271" t="n">
         <v>6</v>
@@ -42188,7 +42188,7 @@
         <v>750</v>
       </c>
       <c r="AC271" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD271" t="n">
         <v>30</v>
@@ -42484,7 +42484,7 @@
         <v>750</v>
       </c>
       <c r="Y273" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z273" t="n">
         <v>6</v>
@@ -42496,7 +42496,7 @@
         <v>750</v>
       </c>
       <c r="AC273" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD273" t="n">
         <v>30</v>
@@ -42792,7 +42792,7 @@
         <v>500</v>
       </c>
       <c r="Y275" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z275" t="n">
         <v>4</v>
@@ -42804,7 +42804,7 @@
         <v>500</v>
       </c>
       <c r="AC275" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD275" t="n">
         <v>30</v>
@@ -43100,7 +43100,7 @@
         <v>500</v>
       </c>
       <c r="Y277" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z277" t="n">
         <v>4</v>
@@ -43112,7 +43112,7 @@
         <v>500</v>
       </c>
       <c r="AC277" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD277" t="n">
         <v>30</v>
@@ -43408,7 +43408,7 @@
         <v>500</v>
       </c>
       <c r="Y279" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z279" t="n">
         <v>4</v>
@@ -43420,7 +43420,7 @@
         <v>500</v>
       </c>
       <c r="AC279" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD279" t="n">
         <v>30</v>
@@ -43716,7 +43716,7 @@
         <v>500</v>
       </c>
       <c r="Y281" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="Z281" t="n">
         <v>4</v>
@@ -43728,7 +43728,7 @@
         <v>500</v>
       </c>
       <c r="AC281" t="n">
-        <v>25.97</v>
+        <v>20</v>
       </c>
       <c r="AD281" t="n">
         <v>30</v>
@@ -44024,7 +44024,7 @@
         <v>750</v>
       </c>
       <c r="Y283" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z283" t="n">
         <v>6</v>
@@ -44036,7 +44036,7 @@
         <v>750</v>
       </c>
       <c r="AC283" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD283" t="n">
         <v>30</v>
@@ -44332,7 +44332,7 @@
         <v>750</v>
       </c>
       <c r="Y285" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z285" t="n">
         <v>6</v>
@@ -44344,7 +44344,7 @@
         <v>750</v>
       </c>
       <c r="AC285" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD285" t="n">
         <v>30</v>
@@ -44640,7 +44640,7 @@
         <v>750</v>
       </c>
       <c r="Y287" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z287" t="n">
         <v>6</v>
@@ -44652,7 +44652,7 @@
         <v>750</v>
       </c>
       <c r="AC287" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD287" t="n">
         <v>30</v>
@@ -44948,7 +44948,7 @@
         <v>750</v>
       </c>
       <c r="Y289" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="Z289" t="n">
         <v>6</v>
@@ -44960,7 +44960,7 @@
         <v>750</v>
       </c>
       <c r="AC289" t="n">
-        <v>51.95</v>
+        <v>40</v>
       </c>
       <c r="AD289" t="n">
         <v>30</v>
@@ -45256,7 +45256,7 @@
         <v>1000</v>
       </c>
       <c r="Y291" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z291" t="n">
         <v>8</v>
@@ -45268,7 +45268,7 @@
         <v>1000</v>
       </c>
       <c r="AC291" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD291" t="n">
         <v>30</v>
@@ -45564,7 +45564,7 @@
         <v>1000</v>
       </c>
       <c r="Y293" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z293" t="n">
         <v>8</v>
@@ -45576,7 +45576,7 @@
         <v>1000</v>
       </c>
       <c r="AC293" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD293" t="n">
         <v>30</v>
@@ -45872,7 +45872,7 @@
         <v>1000</v>
       </c>
       <c r="Y295" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z295" t="n">
         <v>8</v>
@@ -45884,7 +45884,7 @@
         <v>1000</v>
       </c>
       <c r="AC295" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD295" t="n">
         <v>30</v>
@@ -46180,7 +46180,7 @@
         <v>1000</v>
       </c>
       <c r="Y297" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z297" t="n">
         <v>8</v>
@@ -46192,7 +46192,7 @@
         <v>1000</v>
       </c>
       <c r="AC297" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD297" t="n">
         <v>30</v>
@@ -46488,7 +46488,7 @@
         <v>1000</v>
       </c>
       <c r="Y299" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z299" t="n">
         <v>8</v>
@@ -46500,7 +46500,7 @@
         <v>1000</v>
       </c>
       <c r="AC299" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD299" t="n">
         <v>30</v>
@@ -46796,7 +46796,7 @@
         <v>1000</v>
       </c>
       <c r="Y301" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z301" t="n">
         <v>8</v>
@@ -46808,7 +46808,7 @@
         <v>1000</v>
       </c>
       <c r="AC301" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD301" t="n">
         <v>30</v>
@@ -47104,7 +47104,7 @@
         <v>1000</v>
       </c>
       <c r="Y303" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z303" t="n">
         <v>8</v>
@@ -47116,7 +47116,7 @@
         <v>1000</v>
       </c>
       <c r="AC303" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD303" t="n">
         <v>30</v>
@@ -47412,7 +47412,7 @@
         <v>1000</v>
       </c>
       <c r="Y305" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="Z305" t="n">
         <v>8</v>
@@ -47424,7 +47424,7 @@
         <v>1000</v>
       </c>
       <c r="AC305" t="n">
-        <v>77.92</v>
+        <v>60</v>
       </c>
       <c r="AD305" t="n">
         <v>30</v>
@@ -47720,7 +47720,7 @@
         <v>850</v>
       </c>
       <c r="Y307" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z307" t="n">
         <v>7</v>
@@ -47732,7 +47732,7 @@
         <v>850</v>
       </c>
       <c r="AC307" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD307" t="n">
         <v>30</v>
@@ -48028,7 +48028,7 @@
         <v>850</v>
       </c>
       <c r="Y309" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z309" t="n">
         <v>7</v>
@@ -48040,7 +48040,7 @@
         <v>850</v>
       </c>
       <c r="AC309" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD309" t="n">
         <v>30</v>
@@ -48336,7 +48336,7 @@
         <v>850</v>
       </c>
       <c r="Y311" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z311" t="n">
         <v>7</v>
@@ -48348,7 +48348,7 @@
         <v>850</v>
       </c>
       <c r="AC311" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD311" t="n">
         <v>30</v>
@@ -48644,7 +48644,7 @@
         <v>850</v>
       </c>
       <c r="Y313" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="Z313" t="n">
         <v>7</v>
@@ -48656,7 +48656,7 @@
         <v>850</v>
       </c>
       <c r="AC313" t="n">
-        <v>64.94</v>
+        <v>50</v>
       </c>
       <c r="AD313" t="n">
         <v>30</v>
@@ -48952,7 +48952,7 @@
         <v>625</v>
       </c>
       <c r="Y315" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z315" t="n">
         <v>5</v>
@@ -48964,7 +48964,7 @@
         <v>625</v>
       </c>
       <c r="AC315" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD315" t="n">
         <v>30</v>
@@ -49260,7 +49260,7 @@
         <v>625</v>
       </c>
       <c r="Y317" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z317" t="n">
         <v>5</v>
@@ -49272,7 +49272,7 @@
         <v>625</v>
       </c>
       <c r="AC317" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD317" t="n">
         <v>30</v>
@@ -49568,7 +49568,7 @@
         <v>625</v>
       </c>
       <c r="Y319" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z319" t="n">
         <v>5</v>
@@ -49580,7 +49580,7 @@
         <v>625</v>
       </c>
       <c r="AC319" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD319" t="n">
         <v>30</v>
@@ -49876,7 +49876,7 @@
         <v>625</v>
       </c>
       <c r="Y321" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="Z321" t="n">
         <v>5</v>
@@ -49888,7 +49888,7 @@
         <v>625</v>
       </c>
       <c r="AC321" t="n">
-        <v>38.96</v>
+        <v>30</v>
       </c>
       <c r="AD321" t="n">
         <v>30</v>

</xml_diff>